<commit_message>
add wbs, fix text format
</commit_message>
<xml_diff>
--- a/invoice_automation/clients/northsky_comm/templates/SupplierLists.xlsx
+++ b/invoice_automation/clients/northsky_comm/templates/SupplierLists.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\PYTHON\PDFInvoiceExtract\invoice_automation\clients\northsky_comm\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{515AB130-0E5E-44E5-838A-1740F6EC6521}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62B85741-5F11-45E9-94CF-0DC277C6FC79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9510" yWindow="-90" windowWidth="19380" windowHeight="10260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9510" yWindow="-90" windowWidth="19380" windowHeight="10260" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="VENDORS" sheetId="1" r:id="rId1"/>

</xml_diff>